<commit_message>
feat: 20 faction units get own art (HoMM2 + custom Treant/Drow)
Extracted 16 unit icons from HoMM2 Units.gif sheet (Dwarf, Priest,
Crusader, Templar, Druid, Apprentice, Crystal Golem, Djinn, Vampire,
Bone Golem, Goblin, Orc, Ogre, Troll). Custom art for Treant and Drow.
War Mage / Arch Mage reuse SPRITE_MAGE art. All units now have own
SPRITE + ICON TGAs, SPRs built, CSV updated. Audit: 64 PASS, 0 FAIL.
</commit_message>
<xml_diff>
--- a/mom_dimension_inventory.xlsx
+++ b/mom_dimension_inventory.xlsx
@@ -72276,7 +72276,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>SPRITE_MAGE</t>
+          <t>SPRITE_WAR_MAGE</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -72363,7 +72363,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>SPRITE_WARLOCK</t>
+          <t>SPRITE_ARCH_MAGE</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -72450,7 +72450,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>SPRITE_IRON_GOLEM</t>
+          <t>SPRITE_DWARF_WARRIOR</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -72537,7 +72537,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>SPRITE_CATAPULT</t>
+          <t>SPRITE_DWARF_CROSSBOW</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -72624,7 +72624,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>SPRITE_IRON_GOLEM</t>
+          <t>SPRITE_DWARF_RUNESMITH</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -72711,7 +72711,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>SPRITE_GUARDIAN_SPIRIT</t>
+          <t>SPRITE_PRIEST</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -72798,7 +72798,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>SPRITE_KNIGHTS</t>
+          <t>SPRITE_CRUSADER</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -72885,7 +72885,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>SPRITE_PALADINS</t>
+          <t>SPRITE_TEMPLAR</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -72972,7 +72972,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>SPRITE_WAR_MAMMOTH</t>
+          <t>SPRITE_TREANT</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -73059,7 +73059,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>SPRITE_MAGE</t>
+          <t>SPRITE_DRUID</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -73146,7 +73146,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>SPRITE_PHANTOM_WARRIORS</t>
+          <t>SPRITE_APPRENTICE</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -73233,7 +73233,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>SPRITE_IRON_GOLEM</t>
+          <t>SPRITE_CRYSTAL_GOLEM</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -73320,7 +73320,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>SPRITE_AIR_ELEMENTAL</t>
+          <t>SPRITE_DJINN</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -73407,7 +73407,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>SPRITE_WRAITH</t>
+          <t>SPRITE_VAMPIRE</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -73494,7 +73494,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>SPRITE_IRON_GOLEM</t>
+          <t>SPRITE_BONE_GOLEM</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -73581,7 +73581,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>SPRITE_MINION</t>
+          <t>SPRITE_GOBLIN</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -73668,7 +73668,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>SPRITE_MINOTAUR</t>
+          <t>SPRITE_ORC</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -73755,7 +73755,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>SPRITE_WAR_TROLL</t>
+          <t>SPRITE_OGRE</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -73842,7 +73842,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>SPRITE_WAR_TROLL</t>
+          <t>SPRITE_TROLL</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -73929,7 +73929,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>SPRITE_DEMON</t>
+          <t>SPRITE_DROW</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">

</xml_diff>